<commit_message>
Update orders API, server config and add OpenAPI docs
</commit_message>
<xml_diff>
--- a/OrdersProPanel.xlsx
+++ b/OrdersProPanel.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2885" uniqueCount="741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2886" uniqueCount="741">
   <si>
     <t>Domain</t>
   </si>
@@ -32247,7 +32247,9 @@
       <c r="AM416" s="11"/>
       <c r="AN416" s="11"/>
       <c r="AO416" s="11"/>
-      <c r="AP416" s="11"/>
+      <c r="AP416" s="11" t="s">
+        <v>359</v>
+      </c>
     </row>
     <row r="417" spans="1:42" ht="15.75" customHeight="1">
       <c r="A417" s="11"/>

</xml_diff>